<commit_message>
Add Appendix 7 on the source of the k = +2 term of Figure 2
Splits the wildfire damage by the half of the year in which the fire
begins, re-dates the November and December fires to the year after,
builds an alternative shock from the fire-line loss ratio of the state
market, and adds exposure x the state's average damage as a control.
Reports the dating of the Storm Events records, the autocorrelation of
the damage series and each dynamic term estimated on its own.

Also moves the data into 1_data, where the script reads it, and carries
the industry file in six pieces because the zip is over the 100 MB a
file may be on GitHub.
</commit_message>
<xml_diff>
--- a/output/tables_and_figures.xlsx
+++ b/output/tables_and_figures.xlsx
@@ -22,9 +22,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix 4" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix 5" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix 6" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure 1" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure 2" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure 3" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix 7" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure 1" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure 2" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure 3" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -261,6 +262,36 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8953500" cy="3581400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
@@ -285,7 +316,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -340,7 +371,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -684,7 +715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -888,45 +919,57 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Figure 1</t>
+          <t>Appendix 7</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Placebo tests</t>
+          <t>Where the term at k = +2 of Figure 2 comes from, with Figure 4</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Figure 2</t>
+          <t>Figure 1</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Dynamic effect</t>
+          <t>Placebo tests</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>Figure 2</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Dynamic effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
           <t>Figure 3</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Checks on the dynamic effect</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-    </row>
-    <row r="23" ht="62" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+    </row>
+    <row r="24" ht="62" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Sample: insurer × state × year, 38 insurer groups linked to Violation Tracker, 51 states (including DC), 2013-2024. Data: S&amp;P Capital IQ statutory premiums and losses; Violation Tracker penalties; NOAA Storm Events property and crop damage (USD of 2024). All regressions are OLS; standard errors are clustered by insurer unless stated otherwise. In every regression with an interaction, its lower-order terms are included and reported, unless the fixed effects absorb them. Each table states its own sample.</t>
         </is>
@@ -934,9 +977,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A23:B23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -13814,6 +13857,702 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:F60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Appendix 7. Where the term at k = +2 of Figure 2 comes from</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Three things could put a coefficient on damage that arrives after the violations: the dating of the damage, the persistence of wildfire damage within a state, and the sorting of exposed insurers into fire-prone states. The panels take them in that order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Panel A. The dating of the damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>NOAA Storm Events wildfire records</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Wildfire records, 2013-2024</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>3,901</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Records carrying damage</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>840</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Records whose end year differs from the begin year</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Share of the damage, fires beginning January to June</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>0.045</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Share of the damage, fires beginning July to October</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>0.323</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Share of the damage, fires beginning November and December</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>0.631</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Share of the damage, the two largest records</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>0.745</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Panel B. The persistence of wildfire damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Autocorrelation within the state</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Lag 1</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Lag 2</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Lag 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Ln wildfire damage</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>0.441</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>0.416</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>0.464</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Any damage</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>0.457</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>0.436</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>0.456</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Exposure × damage(t+k), number of violations</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Correlation with k = 0</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Estimated on its own</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>In one regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>k = -3</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>0.523</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>-0.1420</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>-0.1034</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>k = -2</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>0.449</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>0.0583</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>0.0820</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>k = -1</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>0.536</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>-0.0058</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>-0.0301</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>k = 0</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>0.1671</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>0.1733**</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>k = +1</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>0.531</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>-0.1197</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>-0.0765</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>k = +2</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>0.464</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>0.1054**</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>0.1194**</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>k = +3</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>0.560</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>0.0505</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>0.0530</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Panel C. The damage measure</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>k = 0</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>k = 0 significant</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>k = +2</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>k = +2 significant</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Ln wildfire damage (Figure 2)</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>0.1733** (0.0834)</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>11 / 12</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>0.1194** (0.0467)</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>11 / 12</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>9,233</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Fires beginning July to December</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>0.0625 (0.0980)</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>0 / 12</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>0.1119** (0.0431)</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>9 / 12</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>9,233</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Fires beginning January to June</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>0.3832** (0.1447)</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>12 / 12</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>0.0665 (0.0688)</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>0 / 12</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>9,233</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>November and December fires dated to the year after</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>0.1679 (0.1002)</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>1 / 12</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>0.0947 (0.0575)</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>7 / 12</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>9,233</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Fire-line loss ratio of the state market</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>0.7612 (0.6278)</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>0 / 12</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>0.3582*** (0.1060)</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>12 / 12</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>6,059</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n"/>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Panel D. Exposure × the state's average damage, added to Figure 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="3" t="inlineStr"/>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>k = 0</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>k = 0 significant</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>k = +2</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>k = +2 significant</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Exposure × the state's average damage</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>0.1602* (0.0810)</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>10 / 12</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>0.1066** (0.0442)</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>11 / 12</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>9,233</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n"/>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+    </row>
+    <row r="60" ht="116" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Notes: Panel A counts the wildfire records of NOAA Storm Events, each dated by the month in which the fire begins; a record whose fire ran across a year end would carry its damage in the earlier year, and none does, so the shares below it are what the annual dating leaves open. Panel B takes the damage of Figure 2: the first column is the correlation of exposure × damage(t+k) with exposure × damage(t) over the sample of Figure 2, the second estimates that term alone on the same sample, and the third repeats the joint estimate of Figure 2. Panels C and D re-estimate Figure 2 under insurer × state and state × year effects; the coefficient columns are the number of violations with a window of plus or minus three years and exposure in year t, and the counts are over all twelve panels of Figure 2 at the 5% level. The two half-year series split the damage of a state and year by the month in which the fire begins, so they sum to the damage of Figure 2; the loss-ratio shock is observed for 2014-2023 only and its window is correspondingly shorter. Every estimate is in output/appendix7_checks.csv. Standard errors clustered by insurer in parentheses. *** p&lt;0.01, ** p&lt;0.05, * p&lt;0.1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A60:F60"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -14247,7 +14986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16183,7 +16922,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>